<commit_message>
Organisation : list page
</commit_message>
<xml_diff>
--- a/sekoya-back/src/main/resources/init/business_data.xlsx
+++ b/sekoya-back/src/main/resources/init/business_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Documents\sekoya\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45BCE2B8-A41B-4E91-A3F8-FC144845C63D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA0A6DD2-901A-4883-B667-BFB61B16671B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25995" windowHeight="12840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="10845" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Role" sheetId="1" r:id="rId1"/>
@@ -89,9 +89,6 @@
     <t>Benichou</t>
   </si>
   <si>
-    <t>GLOBAL_USER_READ,GLOBAL_USER_WRITE,GLOBAL_REFERENCE_DATA_READ,GLOBAL_REFERENCE_DATA_WRITE,GLOBAL_ANNOUNCEMENT_READ,GLOBAL_ANNOUNCEMENT_WRITE</t>
-  </si>
-  <si>
     <t>Organisation</t>
   </si>
   <si>
@@ -135,6 +132,9 @@
   </si>
   <si>
     <t>enumKey</t>
+  </si>
+  <si>
+    <t>GLOBAL_ORGANISATION_READ,GLOBAL_ORGANISATION_WRITE,GLOBAL_USER_READ,GLOBAL_USER_WRITE,GLOBAL_REFERENCE_DATA_READ,GLOBAL_REFERENCE_DATA_WRITE,GLOBAL_ANNOUNCEMENT_READ,GLOBAL_ANNOUNCEMENT_WRITE</t>
   </si>
 </sst>
 </file>
@@ -353,7 +353,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -364,13 +364,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
         <v>30</v>
       </c>
-      <c r="C2" t="s">
-        <v>31</v>
-      </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -378,10 +378,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -455,13 +455,13 @@
         <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G2" t="s">
         <v>15</v>
@@ -470,7 +470,7 @@
         <v>16</v>
       </c>
       <c r="I2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -478,19 +478,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" t="s">
-        <v>24</v>
-      </c>
       <c r="D3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
         <v>21</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" t="s">
-        <v>22</v>
       </c>
       <c r="G3" t="s">
         <v>15</v>
@@ -499,7 +499,7 @@
         <v>16</v>
       </c>
       <c r="I3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -516,13 +516,13 @@
         <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G4" t="s">
         <v>15</v>
@@ -531,7 +531,7 @@
         <v>16</v>
       </c>
       <c r="I4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -542,19 +542,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
         <v>26</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="E5" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G5" t="s">
         <v>15</v>
@@ -563,7 +563,7 @@
         <v>16</v>
       </c>
       <c r="I5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J5">
         <v>1</v>

</xml_diff>

<commit_message>
Processus liste + saisie
</commit_message>
<xml_diff>
--- a/sekoya-back/src/main/resources/init/business_data.xlsx
+++ b/sekoya-back/src/main/resources/init/business_data.xlsx
@@ -45,7 +45,7 @@
     <t xml:space="preserve">ADMINISTRATEUR_FONCTIONNEL</t>
   </si>
   <si>
-    <t xml:space="preserve">GLOBAL_ORGANISATION_READ,GLOBAL_ORGANISATION_WRITE,GLOBAL_SITE_READ,GLOBAL_SITE_WRITE,GLOBAL_USER_READ,GLOBAL_USER_WRITE,GLOBAL_REFERENCE_DATA_READ,GLOBAL_REFERENCE_DATA_WRITE,GLOBAL_ANNOUNCEMENT_READ,GLOBAL_ANNOUNCEMENT_WRITE</t>
+    <t xml:space="preserve">GLOBAL_ORGANISATION_READ,GLOBAL_ORGANISATION_WRITE,GLOBAL_SITE_READ,GLOBAL_SITE_WRITE,GLOBAL_PROCESSUS_READ,GLOBAL_PROCESSUS_WRITE,GLOBAL_USER_READ,GLOBAL_USER_WRITE,GLOBAL_REFERENCE_DATA_READ,GLOBAL_REFERENCE_DATA_WRITE,GLOBAL_ANNOUNCEMENT_READ,GLOBAL_ANNOUNCEMENT_WRITE</t>
   </si>
   <si>
     <t xml:space="preserve">Organisation</t>
@@ -142,7 +142,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -163,11 +163,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -226,7 +221,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
@@ -235,19 +230,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -481,50 +476,50 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="26.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="82.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="26.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="82.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -547,17 +542,17 @@
   <dimension ref="A1:J16"/>
   <sheetFormatPr defaultColWidth="10.71484375" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="32.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="25.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="7.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="244" min="11" style="0" width="10.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="22.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="244" min="11" style="1" width="10.29"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -593,13 +588,13 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>20</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -608,27 +603,27 @@
       <c r="E2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -637,30 +632,30 @@
       <c r="E3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="I3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="0" t="n">
+      <c r="J3" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -669,30 +664,30 @@
       <c r="E4" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="H4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="I4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="0" t="n">
+      <c r="J4" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>34</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -701,19 +696,19 @@
       <c r="E5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="H5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="I5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="0" t="n">
+      <c r="J5" s="1" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>